<commit_message>
fix(practice-paper): correct APJ GAT Mock 5 Q46 key A->B (rearrangement re-derivation)
Q46 (Sentence Rearrangement) was keyed PSRQ (A); the only coherent dialogue
order is QPSR (B) — the peasant's "Yes" (Q) answers the traveller's "Can you...?"
(S1); PSRQ left Q dangling. Flipped the option is_correct flags + recomputed
content_hash on the live PUBLIC row (key change alters the hash). Records file +
OMR Excel updated. The other 6 low-confidence keys re-verified and stand.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/generated-papers/Tags_NDA_APJ_GAT_Mock_5.xlsx
+++ b/generated-papers/Tags_NDA_APJ_GAT_Mock_5.xlsx
@@ -2594,10 +2594,10 @@
         <v>QSRP</v>
       </c>
       <c r="J47" t="str">
-        <v>A</v>
+        <v>B</v>
       </c>
       <c r="K47" t="str">
-        <v>After the traveller asks for an inn (S1), the peasant clarifies (P), the traveller confirms (S), and the peasant gives directions (R) before the closing thanks. Matches option A.</v>
+        <v>Dialogue order: the traveller asks whether the peasant can help (S1); the peasant replies 'Yes' (Q); the peasant then asks whether he wants an inn to spend the night in (P); the traveller replies 'Yes' (S); the peasant gives the directions (R); the traveller thanks him (S6). Sequence QPSR. Matches option B.</v>
       </c>
       <c r="L47" t="str">
         <v>Moderate</v>

</xml_diff>